<commit_message>
replace units initial commit
</commit_message>
<xml_diff>
--- a/pyDGII.extension/pyDGII.tab/Room Location.xlsx
+++ b/pyDGII.extension/pyDGII.tab/Room Location.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\psrimal\Desktop\Diryah Automation\prakritisrimal-automation\pyDGII.extension\pyDGII.tab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D9B7151-FEEF-49B0-924E-FD08E32859DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{705297E9-DC59-44B3-9587-F62CEF89F98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{9A33F726-253C-4876-8A5E-08E5F7D09A43}"/>
+    <workbookView xWindow="4005" yWindow="525" windowWidth="21600" windowHeight="12645" activeTab="1" xr2:uid="{D9C6939E-4F1F-4752-AD36-03712978EDE1}"/>
   </bookViews>
   <sheets>
     <sheet name="Room Location" sheetId="1" r:id="rId1"/>
-    <sheet name="File Location" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="53">
   <si>
     <t xml:space="preserve">Room Name </t>
   </si>
@@ -29,28 +29,157 @@
     <t>Room Location</t>
   </si>
   <si>
-    <t>T1-1</t>
-  </si>
-  <si>
-    <t>1043.578,299.1616,52.1654</t>
-  </si>
-  <si>
-    <t>1072.9415,299.1616,52.1654</t>
-  </si>
-  <si>
-    <t>T2-2B-A1</t>
-  </si>
-  <si>
-    <t>C:\Users\psrimal\Desktop\TYPE2- 2 Bedroom_detached.rvt</t>
-  </si>
-  <si>
-    <t>1205.3234,516.8454,16.7323</t>
-  </si>
-  <si>
-    <t>1559.6541,546.3731,16.7323</t>
-  </si>
-  <si>
-    <t xml:space="preserve">File Location </t>
+    <t>T1-1B-A1</t>
+  </si>
+  <si>
+    <t>1014.0505,353.7926,52.1654</t>
+  </si>
+  <si>
+    <t>1043.414,353.7877,52.1654</t>
+  </si>
+  <si>
+    <t>1072.9415,353.7877,52.1654</t>
+  </si>
+  <si>
+    <t>1545.5465,353.7877,52.1654</t>
+  </si>
+  <si>
+    <t>1574.91,353.7877,52.1654</t>
+  </si>
+  <si>
+    <t>1604.6016,353.7926,52.1654</t>
+  </si>
+  <si>
+    <t>1043.578,298.6694,52.1654</t>
+  </si>
+  <si>
+    <t>1072.9415,298.6694,52.1654</t>
+  </si>
+  <si>
+    <t>1545.5465,298.6694,52.1654</t>
+  </si>
+  <si>
+    <t>1574.91,298.6694,52.1654</t>
+  </si>
+  <si>
+    <t>1456.9638,627.2066,40.3543</t>
+  </si>
+  <si>
+    <t>1486.3274,627.2066,40.3543</t>
+  </si>
+  <si>
+    <t>1575.0741,627.2066,40.3543</t>
+  </si>
+  <si>
+    <t>1604.4376,627.2066,40.3543</t>
+  </si>
+  <si>
+    <t>1456.9638,627.246,28.5433</t>
+  </si>
+  <si>
+    <t>1486.3274,627.246,28.5433</t>
+  </si>
+  <si>
+    <t>1575.0741,627.2458,28.5433</t>
+  </si>
+  <si>
+    <t>1604.4376,627.2458,28.5433</t>
+  </si>
+  <si>
+    <t>1309.326,353.7877,52.1654</t>
+  </si>
+  <si>
+    <t>1338.6896,353.7877,52.1654</t>
+  </si>
+  <si>
+    <t>1309.326,298.7768,52.1654</t>
+  </si>
+  <si>
+    <t>1338.6896,298.6694,52.1654</t>
+  </si>
+  <si>
+    <t>T1-ST-A</t>
+  </si>
+  <si>
+    <t>1053.4205,656.1173,4.9213</t>
+  </si>
+  <si>
+    <t>1131.9966,656.1173,4.9213</t>
+  </si>
+  <si>
+    <t>1171.5308,656.1173,4.9213</t>
+  </si>
+  <si>
+    <t>1013.8864,656.1173,4.9213</t>
+  </si>
+  <si>
+    <t>1191.0518,353.7877,52.1654</t>
+  </si>
+  <si>
+    <t>1161.6883,353.7877,52.1654</t>
+  </si>
+  <si>
+    <t>1161.5828,298.6694,52.1654</t>
+  </si>
+  <si>
+    <t>1191.0518,298.6694,52.1654</t>
+  </si>
+  <si>
+    <t>1014.0505,656.1173,52.1654</t>
+  </si>
+  <si>
+    <t>1043.414,656.1173,52.1654</t>
+  </si>
+  <si>
+    <t>1043.414,600.9991,52.1654</t>
+  </si>
+  <si>
+    <t>1014.0505,601.004,52.1654</t>
+  </si>
+  <si>
+    <t>1132.1607,600.9941,52.1654</t>
+  </si>
+  <si>
+    <t>1161.5242,600.9991,52.1654</t>
+  </si>
+  <si>
+    <t>1250.2709,600.9991,52.1654</t>
+  </si>
+  <si>
+    <t>1279.6344,601.004,52.1654</t>
+  </si>
+  <si>
+    <t>1279.6344,656.1173,52.1654</t>
+  </si>
+  <si>
+    <t>1250.1725,656.1173,52.1654</t>
+  </si>
+  <si>
+    <t>1161.5242,656.1173,52.1654</t>
+  </si>
+  <si>
+    <t>1131.9967,656.1173,52.1654</t>
+  </si>
+  <si>
+    <t>1427.4363,353.7877,52.1654</t>
+  </si>
+  <si>
+    <t>1456.7998,353.7877,52.1654</t>
+  </si>
+  <si>
+    <t>1456.7998,298.6694,52.1654</t>
+  </si>
+  <si>
+    <t>1427.4363,298.6694,52.1654</t>
+  </si>
+  <si>
+    <t>File Location</t>
+  </si>
+  <si>
+    <t>P:\_short-term-01\S24107-0100D\OneDrive_2024-05-17 (1)\Revit_WIP\Safdie Typologies\2024.10.23_152_TYPOLOGIES\TYPE 01\T1-ST-A.rvt</t>
+  </si>
+  <si>
+    <t>P:\_short-term-01\S24107-0100D\OneDrive_2024-05-17 (1)\Revit_WIP\Safdie Typologies\2024.10.23_152_TYPOLOGIES\TYPE 01\T1-1B-A1.rvt</t>
   </si>
 </sst>
 </file>
@@ -910,11 +1039,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB245198-2662-418E-8FB5-1CDE94E581E1}">
-  <dimension ref="A1:B5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B774BB5E-FC1A-4400-9CC5-6094DC525821}">
+  <dimension ref="A1:B47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="28.42578125" customWidth="1"/>
+    <col min="1" max="1" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -943,18 +1072,354 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>2</v>
+      </c>
+      <c r="B17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>2</v>
+      </c>
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>2</v>
+      </c>
+      <c r="B20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>2</v>
+      </c>
+      <c r="B22" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>2</v>
+      </c>
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>2</v>
+      </c>
+      <c r="B29" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>2</v>
+      </c>
+      <c r="B30" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>2</v>
+      </c>
+      <c r="B31" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>2</v>
+      </c>
+      <c r="B32" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>2</v>
+      </c>
+      <c r="B34" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>2</v>
+      </c>
+      <c r="B35" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>2</v>
+      </c>
+      <c r="B36" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>2</v>
+      </c>
+      <c r="B37" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>2</v>
+      </c>
+      <c r="B38" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>2</v>
+      </c>
+      <c r="B39" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>2</v>
+      </c>
+      <c r="B40" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>2</v>
+      </c>
+      <c r="B41" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>2</v>
+      </c>
+      <c r="B42" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>2</v>
+      </c>
+      <c r="B43" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>2</v>
+      </c>
+      <c r="B44" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>2</v>
+      </c>
+      <c r="B45" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B46" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>2</v>
+      </c>
+      <c r="B47" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -963,28 +1428,32 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F62468D3-C4C1-4A2D-84C1-60F41DF6841F}">
-  <dimension ref="A1:B2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC90F6EF-C0A0-4721-8174-4EF8CD3E75A0}">
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.85546875" customWidth="1"/>
-    <col min="2" max="2" width="37.85546875" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>